<commit_message>
import techs from a year to another
</commit_message>
<xml_diff>
--- a/case_studies/2050/technologies.xlsx
+++ b/case_studies/2050/technologies.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Github\AdOpT-NET0_my\case_studies\2050\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C6BDA0F-FBDF-4836-8A32-04BEC6B77DDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_FDB96DFE34A4133CF4515CD4235BDA1626C6A626" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -676,7 +676,7 @@
         <v>0</v>
       </c>
       <c r="F2" s="3">
-        <v>17.75</v>
+        <v>6.77</v>
       </c>
       <c r="G2" s="3">
         <v>0</v>
@@ -688,7 +688,7 @@
         <v>0</v>
       </c>
       <c r="J2" s="3">
-        <v>248.31</v>
+        <v>238.79</v>
       </c>
       <c r="K2" s="3">
         <v>0</v>
@@ -706,10 +706,10 @@
         <v>0</v>
       </c>
       <c r="P2" s="3">
-        <v>170.14</v>
+        <v>213.75</v>
       </c>
       <c r="Q2" s="3">
-        <v>218.87</v>
+        <v>262.47000000000003</v>
       </c>
       <c r="R2" s="3">
         <v>0</v>
@@ -727,10 +727,10 @@
         <v>39.340000000000003</v>
       </c>
       <c r="W2" s="3">
-        <v>245.72</v>
+        <v>238.8</v>
       </c>
       <c r="X2" s="3">
-        <v>56.18</v>
+        <v>0</v>
       </c>
       <c r="Y2" s="3">
         <v>0</v>
@@ -739,7 +739,7 @@
         <v>0</v>
       </c>
       <c r="AA2" s="3">
-        <v>2100.29</v>
+        <v>0</v>
       </c>
       <c r="AB2" s="3">
         <v>0</v>
@@ -762,7 +762,7 @@
         <v>0</v>
       </c>
       <c r="C3" s="5">
-        <v>1964.78</v>
+        <v>1964.73</v>
       </c>
       <c r="D3" s="5">
         <v>0</v>
@@ -771,7 +771,7 @@
         <v>0</v>
       </c>
       <c r="F3" s="5">
-        <v>0.03</v>
+        <v>3.18</v>
       </c>
       <c r="G3" s="5">
         <v>0</v>
@@ -834,7 +834,7 @@
         <v>0</v>
       </c>
       <c r="AA3" s="5">
-        <v>1933.26</v>
+        <v>0</v>
       </c>
       <c r="AB3" s="5">
         <v>0</v>
@@ -843,10 +843,10 @@
         <v>0</v>
       </c>
       <c r="AD3" s="5">
-        <v>4.7699999999999996</v>
+        <v>0</v>
       </c>
       <c r="AE3" s="5">
-        <v>30.6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:31" x14ac:dyDescent="0.3">
@@ -866,7 +866,7 @@
         <v>0</v>
       </c>
       <c r="F4" s="3">
-        <v>50.85</v>
+        <v>104.51</v>
       </c>
       <c r="G4" s="3">
         <v>0</v>
@@ -878,13 +878,13 @@
         <v>0</v>
       </c>
       <c r="J4" s="3">
-        <v>389.78</v>
+        <v>343.25</v>
       </c>
       <c r="K4" s="3">
-        <v>64.34</v>
+        <v>158.74</v>
       </c>
       <c r="L4" s="3">
-        <v>38.01</v>
+        <v>135.93</v>
       </c>
       <c r="M4" s="3">
         <v>0</v>
@@ -896,19 +896,19 @@
         <v>0</v>
       </c>
       <c r="P4" s="3">
-        <v>388.71</v>
+        <v>586.46</v>
       </c>
       <c r="Q4" s="3">
-        <v>456.17</v>
+        <v>653.91999999999996</v>
       </c>
       <c r="R4" s="3">
-        <v>380.67</v>
+        <v>346.18</v>
       </c>
       <c r="S4" s="3">
         <v>43.32</v>
       </c>
       <c r="T4" s="3">
-        <v>0</v>
+        <v>128.11000000000001</v>
       </c>
       <c r="U4" s="3">
         <v>0</v>
@@ -917,28 +917,28 @@
         <v>11.05</v>
       </c>
       <c r="W4" s="3">
-        <v>377.67</v>
+        <v>343.17</v>
       </c>
       <c r="X4" s="3">
-        <v>740</v>
+        <v>515.78</v>
       </c>
       <c r="Y4" s="3">
         <v>0</v>
       </c>
       <c r="Z4" s="3">
-        <v>0</v>
+        <v>70.16</v>
       </c>
       <c r="AA4" s="3">
         <v>0</v>
       </c>
       <c r="AB4" s="3">
-        <v>510.85</v>
+        <v>0</v>
       </c>
       <c r="AC4" s="3">
         <v>0</v>
       </c>
       <c r="AD4" s="3">
-        <v>76.28</v>
+        <v>0</v>
       </c>
       <c r="AE4" s="3">
         <v>0</v>
@@ -952,7 +952,7 @@
         <v>0</v>
       </c>
       <c r="C5" s="5">
-        <v>0</v>
+        <v>78.12</v>
       </c>
       <c r="D5" s="5">
         <v>0</v>
@@ -961,7 +961,7 @@
         <v>0</v>
       </c>
       <c r="F5" s="5">
-        <v>0</v>
+        <v>3.13</v>
       </c>
       <c r="G5" s="5">
         <v>0</v>
@@ -976,10 +976,10 @@
         <v>198.78</v>
       </c>
       <c r="K5" s="5">
-        <v>163.36000000000001</v>
+        <v>146.59</v>
       </c>
       <c r="L5" s="5">
-        <v>110.53</v>
+        <v>102.64</v>
       </c>
       <c r="M5" s="5">
         <v>0</v>
@@ -1003,7 +1003,7 @@
         <v>0</v>
       </c>
       <c r="T5" s="5">
-        <v>110.53</v>
+        <v>102.64</v>
       </c>
       <c r="U5" s="5">
         <v>0</v>
@@ -1030,7 +1030,7 @@
         <v>0</v>
       </c>
       <c r="AC5" s="5">
-        <v>601.29999999999995</v>
+        <v>0</v>
       </c>
       <c r="AD5" s="5">
         <v>0</v>
@@ -1044,10 +1044,10 @@
         <v>35</v>
       </c>
       <c r="B6" s="3">
-        <v>469.01</v>
+        <v>0</v>
       </c>
       <c r="C6" s="3">
-        <v>444.62</v>
+        <v>1033.24</v>
       </c>
       <c r="D6" s="3">
         <v>0</v>
@@ -1056,7 +1056,7 @@
         <v>0</v>
       </c>
       <c r="F6" s="3">
-        <v>17.78</v>
+        <v>18.559999999999999</v>
       </c>
       <c r="G6" s="3">
         <v>0</v>
@@ -1068,13 +1068,13 @@
         <v>0</v>
       </c>
       <c r="J6" s="3">
-        <v>113.82</v>
+        <v>98.36</v>
       </c>
       <c r="K6" s="3">
-        <v>0</v>
+        <v>38.26</v>
       </c>
       <c r="L6" s="3">
-        <v>23.14</v>
+        <v>60.58</v>
       </c>
       <c r="M6" s="3">
         <v>0</v>
@@ -1086,19 +1086,19 @@
         <v>0</v>
       </c>
       <c r="P6" s="3">
-        <v>139.33000000000001</v>
+        <v>210.19</v>
       </c>
       <c r="Q6" s="3">
-        <v>139.37</v>
+        <v>210.23</v>
       </c>
       <c r="R6" s="3">
-        <v>116.66</v>
+        <v>105.43</v>
       </c>
       <c r="S6" s="3">
         <v>0</v>
       </c>
       <c r="T6" s="3">
-        <v>0</v>
+        <v>35.369999999999997</v>
       </c>
       <c r="U6" s="3">
         <v>0</v>
@@ -1107,7 +1107,7 @@
         <v>0</v>
       </c>
       <c r="W6" s="3">
-        <v>116.72</v>
+        <v>105.49</v>
       </c>
       <c r="X6" s="3">
         <v>0</v>
@@ -1125,10 +1125,10 @@
         <v>0</v>
       </c>
       <c r="AC6" s="3">
-        <v>1071.04</v>
+        <v>0</v>
       </c>
       <c r="AD6" s="3">
-        <v>21.22</v>
+        <v>0</v>
       </c>
       <c r="AE6" s="3">
         <v>0</v>
@@ -1142,7 +1142,7 @@
         <v>0</v>
       </c>
       <c r="C7" s="5">
-        <v>21.22</v>
+        <v>90.27</v>
       </c>
       <c r="D7" s="5">
         <v>0</v>
@@ -1151,7 +1151,7 @@
         <v>0</v>
       </c>
       <c r="F7" s="5">
-        <v>0</v>
+        <v>5.0199999999999996</v>
       </c>
       <c r="G7" s="5">
         <v>0</v>
@@ -1220,7 +1220,7 @@
         <v>0</v>
       </c>
       <c r="AC7" s="5">
-        <v>22.17</v>
+        <v>0</v>
       </c>
       <c r="AD7" s="5">
         <v>0</v>
@@ -1237,7 +1237,7 @@
         <v>0</v>
       </c>
       <c r="C8" s="3">
-        <v>0</v>
+        <v>1026.06</v>
       </c>
       <c r="D8" s="3">
         <v>0</v>
@@ -1261,10 +1261,10 @@
         <v>0</v>
       </c>
       <c r="K8" s="3">
-        <v>30.42</v>
+        <v>0</v>
       </c>
       <c r="L8" s="3">
-        <v>180.55</v>
+        <v>129.29</v>
       </c>
       <c r="M8" s="3">
         <v>0</v>
@@ -1276,31 +1276,31 @@
         <v>0</v>
       </c>
       <c r="P8" s="3">
-        <v>279.01</v>
+        <v>279.02</v>
       </c>
       <c r="Q8" s="3">
         <v>323.79000000000002</v>
       </c>
       <c r="R8" s="3">
-        <v>0</v>
+        <v>5.52</v>
       </c>
       <c r="S8" s="3">
         <v>30.17</v>
       </c>
       <c r="T8" s="3">
-        <v>143.97</v>
+        <v>92.71</v>
       </c>
       <c r="U8" s="3">
         <v>0</v>
       </c>
       <c r="V8" s="3">
-        <v>1.83</v>
+        <v>1.82</v>
       </c>
       <c r="W8" s="3">
         <v>5.37</v>
       </c>
       <c r="X8" s="3">
-        <v>0</v>
+        <v>136.33000000000001</v>
       </c>
       <c r="Y8" s="3">
         <v>0</v>
@@ -1315,13 +1315,13 @@
         <v>0</v>
       </c>
       <c r="AC8" s="3">
-        <v>519.07000000000005</v>
+        <v>0</v>
       </c>
       <c r="AD8" s="3">
         <v>0</v>
       </c>
       <c r="AE8" s="3">
-        <v>7.15</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1330,7 +1330,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BDE9BCA-3CC4-4E74-8992-63088FB367A4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:AE8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>

</xml_diff>